<commit_message>
Updated Suite.xml to run CalendarTest
</commit_message>
<xml_diff>
--- a/src/test/resources/TestScriptData.xlsx
+++ b/src/test/resources/TestScriptData.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="55">
   <si>
     <t>Event Name</t>
   </si>
@@ -183,6 +183,9 @@
   </si>
   <si>
     <t>Sprint Planning Meeting_0</t>
+  </si>
+  <si>
+    <t>Sprint Planning Meeting_1862</t>
   </si>
 </sst>
 </file>
@@ -1193,7 +1196,7 @@
         <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C2" t="s">
         <v>42</v>
@@ -1407,5 +1410,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>